<commit_message>
Beispielpasswoerter durch Platzhalter ersetzen
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/beispiel_stammliste.xlsx
+++ b/beispiel_stammliste.xlsx
@@ -33,16 +33,16 @@
     <t>Passwort</t>
   </si>
   <si>
-    <t>start7391</t>
-  </si>
-  <si>
-    <t>hafen2048</t>
+    <t>BEISPIEL-Passwort1</t>
+  </si>
+  <si>
+    <t>BEISPIEL-Passwort2</t>
   </si>
   <si>
     <t>00345</t>
   </si>
   <si>
-    <t>wolke5517</t>
+    <t>BEISPIEL-Passwort3</t>
   </si>
   <si>
     <t>000123</t>

</xml_diff>